<commit_message>
Added difficulty specific starting techs
</commit_message>
<xml_diff>
--- a/docs/Logic Requirements/Ageipelago Barbarossa.xlsx
+++ b/docs/Logic Requirements/Ageipelago Barbarossa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefb\OneDrive\Desktop\Logic Requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4780AB0-D514-48BF-B10B-41CFC43C0E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138D7F41-528C-4FFC-9076-4AF12B792ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{3EBDBD80-CAB1-4BA3-AD20-38FC2022F392}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{3EBDBD80-CAB1-4BA3-AD20-38FC2022F392}"/>
   </bookViews>
   <sheets>
     <sheet name="Barbarossa" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="211">
   <si>
     <t>Scenario</t>
   </si>
@@ -4163,12 +4163,54 @@
     <t>No Carvel Hull
 No Spies</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Murder Holes and Herbal Medicine automatically researched for Teutons
+War Galley and Fervor are researched automatically
+On </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Moderate /Standard</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: Sanctity is researched automatically
+On </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Standard</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Redemption is researched automatically</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4401,6 +4443,12 @@
     <font>
       <sz val="14"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -4712,6 +4760,15 @@
     <xf numFmtId="0" fontId="33" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4728,15 +4785,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -5398,11 +5446,11 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="49" t="s">
         <v>200</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="48"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
       <c r="G2" s="2" t="s">
         <v>81</v>
       </c>
@@ -5417,11 +5465,11 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="52" t="s">
         <v>205</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="54"/>
       <c r="G3" s="9" t="s">
         <v>83</v>
       </c>
@@ -5459,13 +5507,13 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="93.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="46" t="s">
         <v>207</v>
       </c>
       <c r="G5" s="9" t="s">
@@ -5482,8 +5530,8 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="20"/>
       <c r="G6" s="9" t="s">
         <v>90</v>
@@ -5499,8 +5547,8 @@
       </c>
     </row>
     <row r="7" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
       <c r="D7" s="20"/>
       <c r="G7" s="12" t="s">
         <v>92</v>
@@ -5516,8 +5564,8 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
       <c r="D8" s="20"/>
       <c r="G8" s="12" t="s">
         <v>96</v>
@@ -5533,8 +5581,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
       <c r="D9" s="20"/>
       <c r="G9" s="12" t="s">
         <v>99</v>
@@ -5550,8 +5598,8 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
       <c r="D10" s="20"/>
       <c r="G10" s="12" t="s">
         <v>128</v>
@@ -5567,8 +5615,8 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="20"/>
       <c r="G11" s="12" t="s">
         <v>125</v>
@@ -5584,8 +5632,8 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
       <c r="D12" s="20"/>
       <c r="G12" s="12" t="s">
         <v>102</v>
@@ -5601,8 +5649,8 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
       <c r="D13" s="20"/>
       <c r="G13" s="39" t="s">
         <v>129</v>
@@ -5618,8 +5666,8 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
       <c r="D14" s="20"/>
       <c r="G14" s="14" t="s">
         <v>111</v>
@@ -5635,8 +5683,8 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
       <c r="D15" s="20"/>
       <c r="G15" s="23" t="s">
         <v>130</v>
@@ -5652,8 +5700,8 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
       <c r="D16" s="20"/>
       <c r="G16" s="23" t="s">
         <v>133</v>
@@ -5905,11 +5953,11 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="49" t="s">
         <v>200</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="48"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
       <c r="G2" s="2" t="s">
         <v>81</v>
       </c>
@@ -5924,11 +5972,11 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="52" t="s">
         <v>205</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="54"/>
       <c r="G3" s="11" t="s">
         <v>83</v>
       </c>
@@ -5966,13 +6014,13 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="93.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="46" t="s">
         <v>207</v>
       </c>
       <c r="G5" s="12" t="s">
@@ -5989,8 +6037,8 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="20"/>
       <c r="G6" s="12" t="s">
         <v>125</v>
@@ -6006,8 +6054,8 @@
       </c>
     </row>
     <row r="7" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
       <c r="D7" s="20"/>
       <c r="G7" s="13" t="s">
         <v>145</v>
@@ -6023,8 +6071,8 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
       <c r="D8" s="20"/>
       <c r="G8" s="12" t="s">
         <v>102</v>
@@ -6040,8 +6088,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
       <c r="D9" s="20"/>
       <c r="G9" s="12" t="s">
         <v>130</v>
@@ -6057,8 +6105,8 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
       <c r="D10" s="20"/>
       <c r="G10" s="12" t="s">
         <v>119</v>
@@ -6074,8 +6122,8 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="20"/>
       <c r="G11" s="24" t="s">
         <v>128</v>
@@ -6091,8 +6139,8 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
       <c r="D12" s="20"/>
       <c r="G12" s="24" t="s">
         <v>134</v>
@@ -6108,8 +6156,8 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
       <c r="D13" s="20"/>
       <c r="G13" s="24" t="s">
         <v>99</v>
@@ -6125,8 +6173,8 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
       <c r="D14" s="20"/>
       <c r="G14" s="15" t="s">
         <v>92</v>
@@ -6142,8 +6190,8 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
       <c r="D15" s="20"/>
       <c r="G15" s="19"/>
       <c r="H15" s="19"/>
@@ -6155,8 +6203,8 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
       <c r="D16" s="20"/>
       <c r="G16" s="27"/>
       <c r="H16" s="27"/>
@@ -6336,11 +6384,11 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="49" t="s">
         <v>200</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="48"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
       <c r="G2" s="2" t="s">
         <v>81</v>
       </c>
@@ -6355,11 +6403,11 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="52" t="s">
         <v>205</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="54"/>
       <c r="G3" s="11" t="s">
         <v>83</v>
       </c>
@@ -6396,15 +6444,15 @@
         <v>84</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="93.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="52" t="s">
+    <row r="5" spans="2:12" ht="337.5" x14ac:dyDescent="0.25">
+      <c r="B5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="D5" s="52" t="s">
-        <v>207</v>
+      <c r="D5" s="46" t="s">
+        <v>210</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>88</v>
@@ -6420,8 +6468,8 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="20"/>
       <c r="G6" s="9" t="s">
         <v>90</v>
@@ -6437,8 +6485,8 @@
       </c>
     </row>
     <row r="7" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
       <c r="D7" s="20"/>
       <c r="G7" s="14" t="s">
         <v>92</v>
@@ -6454,8 +6502,8 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
       <c r="D8" s="20"/>
       <c r="G8" s="14" t="s">
         <v>133</v>
@@ -6471,8 +6519,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
       <c r="D9" s="20"/>
       <c r="G9" s="14" t="s">
         <v>132</v>
@@ -6488,8 +6536,8 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
       <c r="D10" s="20"/>
       <c r="G10" s="14" t="s">
         <v>96</v>
@@ -6505,8 +6553,8 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="20"/>
       <c r="G11" s="14" t="s">
         <v>94</v>
@@ -6522,8 +6570,8 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
       <c r="D12" s="20"/>
       <c r="G12" s="14" t="s">
         <v>102</v>
@@ -6539,8 +6587,8 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
       <c r="D13" s="20"/>
       <c r="G13" s="23" t="s">
         <v>146</v>
@@ -6556,8 +6604,8 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
       <c r="D14" s="20"/>
       <c r="G14" s="23" t="s">
         <v>119</v>
@@ -6573,8 +6621,8 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
       <c r="D15" s="20"/>
       <c r="G15" s="23" t="s">
         <v>111</v>
@@ -6590,8 +6638,8 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
       <c r="D16" s="20"/>
       <c r="G16" s="23" t="s">
         <v>125</v>
@@ -6864,6 +6912,7 @@
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6879,11 +6928,11 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="49" t="s">
         <v>200</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="48"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
       <c r="G2" s="2" t="s">
         <v>81</v>
       </c>
@@ -6898,11 +6947,11 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="52" t="s">
         <v>208</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="54"/>
       <c r="G3" s="11" t="s">
         <v>83</v>
       </c>
@@ -6940,13 +6989,13 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="46" t="s">
         <v>206</v>
       </c>
       <c r="G5" s="9" t="s">
@@ -6963,8 +7012,8 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="20"/>
       <c r="G6" s="9" t="s">
         <v>90</v>
@@ -6980,8 +7029,8 @@
       </c>
     </row>
     <row r="7" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
       <c r="D7" s="20"/>
       <c r="G7" s="24" t="s">
         <v>92</v>
@@ -6997,8 +7046,8 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
       <c r="D8" s="20"/>
       <c r="G8" s="24" t="s">
         <v>96</v>
@@ -7014,8 +7063,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
       <c r="D9" s="20"/>
       <c r="G9" s="24" t="s">
         <v>127</v>
@@ -7031,8 +7080,8 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
       <c r="D10" s="20"/>
       <c r="G10" s="24" t="s">
         <v>134</v>
@@ -7048,8 +7097,8 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="20"/>
       <c r="G11" s="38" t="s">
         <v>104</v>
@@ -7065,8 +7114,8 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
       <c r="D12" s="20"/>
       <c r="G12" s="25" t="s">
         <v>146</v>
@@ -7082,8 +7131,8 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
       <c r="D13" s="20"/>
       <c r="G13" s="25" t="s">
         <v>161</v>
@@ -7099,8 +7148,8 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
       <c r="D14" s="20"/>
       <c r="G14" s="25" t="s">
         <v>119</v>
@@ -7116,8 +7165,8 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
       <c r="D15" s="20"/>
       <c r="G15" s="25" t="s">
         <v>121</v>
@@ -7133,8 +7182,8 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
       <c r="D16" s="20"/>
       <c r="G16" s="25" t="s">
         <v>164</v>
@@ -7398,11 +7447,11 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="49" t="s">
         <v>200</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="48"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
       <c r="G2" s="2" t="s">
         <v>81</v>
       </c>
@@ -7417,11 +7466,11 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="52" t="s">
         <v>208</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="54"/>
       <c r="G3" s="11" t="s">
         <v>83</v>
       </c>
@@ -7459,13 +7508,13 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="46" t="s">
         <v>204</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="46" t="s">
         <v>204</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="46" t="s">
         <v>204</v>
       </c>
       <c r="G5" s="9" t="s">
@@ -7482,8 +7531,8 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="20"/>
       <c r="G6" s="36" t="s">
         <v>175</v>
@@ -7499,8 +7548,8 @@
       </c>
     </row>
     <row r="7" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
       <c r="D7" s="20"/>
       <c r="G7" s="12" t="s">
         <v>163</v>
@@ -7516,8 +7565,8 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
       <c r="D8" s="20"/>
       <c r="G8" s="13" t="s">
         <v>174</v>
@@ -7533,8 +7582,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
       <c r="D9" s="20"/>
       <c r="G9" s="12" t="s">
         <v>165</v>
@@ -7550,8 +7599,8 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
       <c r="D10" s="20"/>
       <c r="G10" s="12" t="s">
         <v>146</v>
@@ -7567,8 +7616,8 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="20"/>
       <c r="G11" s="12" t="s">
         <v>147</v>
@@ -7584,8 +7633,8 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
       <c r="D12" s="20"/>
       <c r="G12" s="12" t="s">
         <v>164</v>
@@ -7601,8 +7650,8 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
       <c r="D13" s="20"/>
       <c r="G13" s="34" t="s">
         <v>132</v>
@@ -7618,8 +7667,8 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
       <c r="D14" s="20"/>
       <c r="G14" s="14" t="s">
         <v>177</v>
@@ -7635,8 +7684,8 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
       <c r="D15" s="20"/>
       <c r="G15" s="14" t="s">
         <v>178</v>
@@ -7652,8 +7701,8 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
       <c r="D16" s="20"/>
       <c r="G16" s="14" t="s">
         <v>141</v>
@@ -7929,11 +7978,11 @@
   <sheetData>
     <row r="1" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="49" t="s">
         <v>200</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="48"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="51"/>
       <c r="G2" s="2" t="s">
         <v>81</v>
       </c>
@@ -7948,11 +7997,11 @@
       </c>
     </row>
     <row r="3" spans="2:12" ht="24" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="52" t="s">
         <v>208</v>
       </c>
-      <c r="C3" s="50"/>
-      <c r="D3" s="51"/>
+      <c r="C3" s="53"/>
+      <c r="D3" s="54"/>
       <c r="G3" s="11" t="s">
         <v>83</v>
       </c>
@@ -7990,13 +8039,13 @@
       </c>
     </row>
     <row r="5" spans="2:12" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="C5" s="52" t="s">
+      <c r="C5" s="46" t="s">
         <v>206</v>
       </c>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="46" t="s">
         <v>209</v>
       </c>
       <c r="G5" s="9" t="s">
@@ -8013,8 +8062,8 @@
       </c>
     </row>
     <row r="6" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="53"/>
-      <c r="C6" s="53"/>
+      <c r="B6" s="47"/>
+      <c r="C6" s="47"/>
       <c r="D6" s="20"/>
       <c r="G6" s="9" t="s">
         <v>90</v>
@@ -8030,8 +8079,8 @@
       </c>
     </row>
     <row r="7" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B7" s="53"/>
-      <c r="C7" s="53"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
       <c r="D7" s="20"/>
       <c r="G7" s="23" t="s">
         <v>92</v>
@@ -8047,8 +8096,8 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="48"/>
       <c r="D8" s="20"/>
       <c r="G8" s="23" t="s">
         <v>165</v>
@@ -8064,8 +8113,8 @@
       </c>
     </row>
     <row r="9" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
       <c r="D9" s="20"/>
       <c r="G9" s="16" t="s">
         <v>190</v>
@@ -8081,8 +8130,8 @@
       </c>
     </row>
     <row r="10" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
       <c r="D10" s="20"/>
       <c r="G10" s="23" t="s">
         <v>114</v>
@@ -8098,8 +8147,8 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B11" s="54"/>
-      <c r="C11" s="54"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
       <c r="D11" s="20"/>
       <c r="G11" s="16" t="s">
         <v>191</v>
@@ -8115,8 +8164,8 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
       <c r="D12" s="20"/>
       <c r="G12" s="14" t="s">
         <v>177</v>
@@ -8132,8 +8181,8 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="47"/>
       <c r="D13" s="20"/>
       <c r="G13" s="14" t="s">
         <v>178</v>
@@ -8149,8 +8198,8 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
       <c r="D14" s="20"/>
       <c r="G14" s="14" t="s">
         <v>141</v>
@@ -8166,8 +8215,8 @@
       </c>
     </row>
     <row r="15" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
+      <c r="B15" s="47"/>
+      <c r="C15" s="47"/>
       <c r="D15" s="20"/>
       <c r="G15" s="39" t="s">
         <v>192</v>
@@ -8183,8 +8232,8 @@
       </c>
     </row>
     <row r="16" spans="2:12" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
       <c r="D16" s="20"/>
       <c r="G16" s="39" t="s">
         <v>194</v>

</xml_diff>